<commit_message>
refactor: Remove DOG_PORTS configuration and update DogAction to use fixed API port 8081
</commit_message>
<xml_diff>
--- a/data/compiled_actions_06-90.xlsx
+++ b/data/compiled_actions_06-90.xlsx
@@ -534,61 +534,61 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-takeoff (3.0)</t>
+takeoff (3.0 s)</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-takeoff (3.0)</t>
+takeoff (3.0 s)</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1)</t>
+move_forward (1.1 s)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1)</t>
+move_forward (1.1 s)</t>
         </is>
       </c>
     </row>
@@ -601,61 +601,61 @@
       <c r="B3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-move_back (3.0)</t>
+move_back (3.0 s)</t>
         </is>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-move_back (3.0)</t>
+move_back (3.0 s)</t>
         </is>
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1)</t>
+move_backward (1.1 s)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1)</t>
+move_backward (1.1 s)</t>
         </is>
       </c>
     </row>
@@ -668,61 +668,61 @@
       <c r="B4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.5 s
-back_fast (4.5)</t>
+back_fast (4.5 s)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.5 s
-back_fast (4.5)</t>
+back_fast (4.5 s)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.5 s
-wave (3.5)</t>
+wave (3.5 s)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1)</t>
+move_forward (1.1 s)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_left (1.1)</t>
+move_left (1.1 s)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1)</t>
+move_forward (1.1 s)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1)</t>
+move_forward (1.1 s)</t>
         </is>
       </c>
     </row>
@@ -735,61 +735,61 @@
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 4.0 s
-bow (4.0)</t>
+bow (4.0 s)</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-land (3.0)</t>
+land (3.0 s)</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
-land (3.0)</t>
+land (3.0 s)</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1)</t>
+move_backward (1.1 s)</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1)</t>
+move_backward (1.1 s)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: Centralize action timing constants in action_times.py and update imports across modules
</commit_message>
<xml_diff>
--- a/data/compiled_actions_06-90.xlsx
+++ b/data/compiled_actions_06-90.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -581,14 +581,14 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1 s)</t>
+          <t>⏱️ TOTAL: 1.0 s
+look_up (1.0 s)</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1 s)</t>
+          <t>⏱️ TOTAL: 1.0 s
+look_up (1.0 s)</t>
         </is>
       </c>
     </row>
@@ -648,148 +648,297 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1 s)</t>
+          <t>⏱️ TOTAL: 1.0 s
+look_down (1.0 s)</t>
         </is>
       </c>
       <c r="K3" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1 s)</t>
+          <t>⏱️ TOTAL: 1.0 s
+look_down (1.0 s)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>69</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 3.5 s
-wave (3.5 s)</t>
+          <t>⏱️ TOTAL: 67.0 s
+dance_seven (67.0 s)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 4.5 s
-back_fast (4.5 s)</t>
+          <t>⏱️ TOTAL: 69.0 s
+dance_six (69.0 s)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 3.5 s
-wave (3.5 s)</t>
+          <t>⏱️ TOTAL: 67.0 s
+dance_seven (67.0 s)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 3.5 s
-wave (3.5 s)</t>
+          <t>⏱️ TOTAL: 67.0 s
+dance_seven (67.0 s)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 4.5 s
-back_fast (4.5 s)</t>
+          <t>⏱️ TOTAL: 69.0 s
+dance_six (69.0 s)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 3.5 s
-wave (3.5 s)</t>
+          <t>⏱️ TOTAL: 67.0 s
+dance_seven (67.0 s)</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1 s)</t>
+          <t>⏱️ TOTAL: 37.50000000000001 s
+move_up_50 (3.0 s)
+move_forward_50 (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_left (1.1 s)</t>
+          <t>⏱️ TOTAL: 37.50000000000001 s
+move_up_50 (3.0 s)
+move_forward_50 (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1 s)</t>
+          <t>⏱️ TOTAL: 39.00000000000001 s
+body_row (2.0 s)
+body_cycle (5.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+rotate (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+bowback (3.0 s)
+move_leftfront (1.1 s)
+move_rightfront (1.1 s)
+move_leftback (1.1 s)
+move_rightback (1.1 s)
+look_rightlower (1.0 s)
+look_leftlower (1.0 s)
+body_cycle (5.0 s)
+balance (0 s)
+height_move (2.0 s)</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_forward (1.1 s)</t>
+          <t>⏱️ TOTAL: 36.00000000000001 s
+body_row (2.0 s)
+balance (0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+rotate (3.0 s)
+move_left (1.1 s)
+move_right (1.1 s)
+move_forward (1.1 s)
+move_back (3.0 s)
+bowback (3.0 s)
+move_leftfront (1.1 s)
+move_rightfront (1.1 s)
+move_leftback (1.1 s)
+move_rightback (1.1 s)
+foreleg_lift (2.0 s)
+backleg_lift (2.0 s)
+body_cycle (5.0 s)
+balance (0 s)
+height_move (2.0 s)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.5 s
+wave (3.5 s)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.5 s
+back_fast (4.5 s)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.5 s
+wave (3.5 s)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.5 s
+wave (3.5 s)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.5 s
+back_fast (4.5 s)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.5 s
+wave (3.5 s)</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 1.1 s
+move_forward (1.1 s)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 1.1 s
+move_left (1.1 s)</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.0 s
+head_ellipse (3.0 s)</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.0 s
+head_ellipse (3.0 s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="G5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 4.0 s
-bow (4.0 s)</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 4.0 s
+bow (4.0 s)</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
 land (3.0 s)</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>⏱️ TOTAL: 3.0 s
 land (3.0 s)</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1 s)</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>⏱️ TOTAL: 1.1 s
-move_backward (1.1 s)</t>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.0 s
+rotate (3.0 s)</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>⏱️ TOTAL: 3.0 s
+rotate (3.0 s)</t>
         </is>
       </c>
     </row>

</xml_diff>